<commit_message>
Mejoras modulos letras, pedidos y despachos
</commit_message>
<xml_diff>
--- a/public/templates/formato_letras.xlsx
+++ b/public/templates/formato_letras.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\juanjhonv\proyects\excelfastify\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\juanjhonv\proyects\api_rest_express\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F4749D3-5865-479D-8758-89AD28B9F959}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28FDB916-B82B-4027-88AB-EDBF973228DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Nº
 Letra</t>
@@ -37,7 +37,11 @@
   </si>
   <si>
     <t>Importe
-Letra</t>
+Letra Soles</t>
+  </si>
+  <si>
+    <t>Importe
+Letra(Dolares)</t>
   </si>
 </sst>
 </file>
@@ -468,16 +472,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D0EB5E5-D857-48B2-A9E2-B2CA43C64BC0}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="57.5" customWidth="1"/>
     <col min="3" max="3" width="38.5" style="8" customWidth="1"/>
     <col min="4" max="4" width="18.875" style="8" customWidth="1"/>
-    <col min="5" max="5" width="14" style="8" customWidth="1"/>
+    <col min="5" max="6" width="14" style="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="24" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -493,47 +497,55 @@
       <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5"/>
+      <c r="F1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="5"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6"/>
       <c r="B2" s="6"/>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
       <c r="E2" s="7"/>
-      <c r="F2" s="6"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="6"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="6"/>
       <c r="B3" s="6"/>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
-      <c r="F3" s="6"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="6"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="6"/>
       <c r="B4" s="6"/>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
       <c r="E4" s="7"/>
-      <c r="F4" s="6"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="6"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6"/>
       <c r="B5" s="6"/>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
       <c r="E5" s="7"/>
-      <c r="F5" s="6"/>
+      <c r="F5" s="7"/>
+      <c r="G5" s="6"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="6"/>
       <c r="B6" s="6"/>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
       <c r="E6" s="7"/>
-      <c r="F6" s="6"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>